<commit_message>
Use exact manufacturer models for all graphics cards
</commit_message>
<xml_diff>
--- a/buildbench-content.xlsx
+++ b/buildbench-content.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="1" r:id="Rf979a80579374b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kategorien" sheetId="2" r:id="Rb193a8e57c1e4519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_case" sheetId="3" r:id="R53693aa443f34e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_motherboard" sheetId="4" r:id="R37d5082167a7499b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_cpu" sheetId="5" r:id="R917d1466925b4975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_gpu" sheetId="6" r:id="R0e20092edef84da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_ram" sheetId="7" r:id="Red0ee38ac0b24d3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_psu" sheetId="8" r:id="R5a903a4bcb60436c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_cooler" sheetId="9" r:id="Rea2b98521d454c8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_storage" sheetId="10" r:id="R82453f3fc54b4286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_standoffs" sheetId="11" r:id="R6b49bc9a35634d11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_screws" sheetId="12" r:id="Rb08a44f44fe34191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_cables" sheetId="13" r:id="Ra4633464ba6c4afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_coolant" sheetId="14" r:id="R2d5ba158dbb649ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lernkarten" sheetId="15" r:id="R1f6f2262b8ce42ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="16" r:id="R2d3699e10fa94801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Netzwerk" sheetId="17" r:id="Re22dfd987a8b4feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mainboard-Netz" sheetId="18" r:id="R9fcc351026004329"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kompatibilität" sheetId="19" r:id="R35eb5cc2d1714b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="1" r:id="R33d30b0e666c4028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kategorien" sheetId="2" r:id="R435c7413f2a34a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_case" sheetId="3" r:id="Rcf5820ef38da4f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_motherboard" sheetId="4" r:id="R4db677926cd84a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_cpu" sheetId="5" r:id="R7c521ee847a142e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_gpu" sheetId="6" r:id="Rdb90d457f3f743b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_ram" sheetId="7" r:id="R1aad7a2b60b94124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_psu" sheetId="8" r:id="R4b665d32121048bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_cooler" sheetId="9" r:id="R7fd97840424a4d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_storage" sheetId="10" r:id="Rc420b0ae56294c24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_standoffs" sheetId="11" r:id="R0934be4eed1f4fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_screws" sheetId="12" r:id="R04148c3c26594654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_cables" sheetId="13" r:id="R8f47bbd32e8c485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_coolant" sheetId="14" r:id="R818d2aadebf14cd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lernkarten" sheetId="15" r:id="Rbe48263ba8644b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="16" r:id="Ra2886fe8228b470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Netzwerk" sheetId="17" r:id="Ree0d293ee0784ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mainboard-Netz" sheetId="18" r:id="R6fd1a54328944bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kompatibilität" sheetId="19" r:id="R11ac0ed9448e40d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,7 +31,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -42,8 +42,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -53,6 +59,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3653"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3653"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3653"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -67,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -75,6 +96,12 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -410,6 +437,11 @@
     <x:col min="10" max="10" width="24" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
     <x:col min="12" max="12" width="24" customWidth="1"/>
+    <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="54" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -473,6 +505,21 @@
           <x:t xml:space="preserve">pcieGen</x:t>
         </x:is>
       </x:c>
+      <x:c r="M1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
+      <x:c r="O1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
+      <x:c r="P1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
+      <x:c r="Q1" s="7" t="str">
+        <x:v>manualUrl</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -533,6 +580,19 @@
       <x:c r="L2" s="2">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="M2" t="str">
+        <x:v>https://www.samsung.com/de/memory-storage/nvme-ssd/990-pro-2tb-nvme-pcie-gen-4-mz-v9p2t0bw/</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>https://download.semiconductor.samsung.com/resources/data-sheet/samsung_nvme_ssd_990_pro_datasheet_rev.2.0.pdf</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>MZ-V9P2T0BW</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q2" t="str"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -593,6 +653,17 @@
       <x:c r="L3" s="2">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://www.sandisk.com/products/ssd/internal-ssd/wd-black-sn850x-nvme-ssd?sku=wds400t2x0e-00bca0</x:v>
+      </x:c>
+      <x:c r="N3" t="str"/>
+      <x:c r="O3" t="str">
+        <x:v>WDS400T2X0E-00BCA0</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q3" t="str"/>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -653,6 +724,19 @@
       <x:c r="L4" s="2">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="M4" t="str">
+        <x:v>https://eu.crucial.com/ssd/t705/ct2000t705ssd3</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>https://eu.crucial.com/content/dam/crucial/ssd-products/t705/flyers/b2c/crucial-t705-b2c-product-flyer-en.pdf</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>CT2000T705SSD3</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q4" t="str"/>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -715,6 +799,19 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
+      <x:c r="M5" t="str">
+        <x:v>https://eu.crucial.com/ssd/mx500/ct2000mx500ssd1</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>https://www.crucial.com/content/dam/crucial/ssd-products/mx500/flyer/crucial-mx500-ssd-productflyer-letter-en.pdf</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>CT2000MX500SSD1</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q5" t="str"/>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
@@ -777,6 +874,19 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
+      <x:c r="M6" t="str">
+        <x:v>https://www.seagate.com/support/internal-hard-drives/nas-drives/ironwolf/</x:v>
+      </x:c>
+      <x:c r="N6" t="str"/>
+      <x:c r="O6" t="str">
+        <x:v>ST8000VN004</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>https://www.seagate.com/www-content/product-content/ironwolf/en-us/docs/100844482b.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="2" t="inlineStr">
@@ -835,6 +945,19 @@
       <x:c r="L7" s="2">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="M7" t="str">
+        <x:v>https://www.samsung.com/uk/memory-storage/nvme-ssd/980-pro-pcle-4-0-nvme-m-2-ssd-1tb-mz-v8p1t0bw/</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>https://image.semiconductor.samsung.com/resources/data-sheet/Samsung-NVMe-SSD-980-PRO-Data-Sheet_Rev.2.1.pdf</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>MZ-V8P1T0BW</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q7" t="str"/>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="2" t="inlineStr">
@@ -893,6 +1016,17 @@
       <x:c r="L8" s="2">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="M8" t="str">
+        <x:v>https://www.samsung.com/uk/memory-storage/nvme-ssd/970-evo-plus-nvme-m-2-ssd-1tb-mz-v7s1t0bw/</x:v>
+      </x:c>
+      <x:c r="N8" t="str"/>
+      <x:c r="O8" t="str">
+        <x:v>MZ-V7S1T0BW</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="Q8" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1786,6 +1920,10 @@
     <x:col min="9" max="9" width="24" customWidth="1"/>
     <x:col min="10" max="10" width="24" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
+    <x:col min="12" max="12" width="54" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1844,6 +1982,18 @@
           <x:t xml:space="preserve">color</x:t>
         </x:is>
       </x:c>
+      <x:c r="L1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="M1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
+      <x:c r="O1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -1899,6 +2049,10 @@
           <x:t xml:space="preserve">transparent</x:t>
         </x:is>
       </x:c>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str"/>
+      <x:c r="N2" t="str"/>
+      <x:c r="O2" t="str"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -1954,6 +2108,16 @@
           <x:t xml:space="preserve">#79dff5</x:t>
         </x:is>
       </x:c>
+      <x:c r="L3" t="str">
+        <x:v>https://shop.alphacool.com/shop/kuehlfluessigkeiten/standard-fluessigkeiten/18651-alphacool-tec-protect-2-clear-1000ml</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://www.alphacool.com/download/DE_1021554_Alphacool_Tec_Protect_2_Clear_1000ml_Datenblatt.pdf</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="O3" t="str"/>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -2009,6 +2173,16 @@
           <x:t xml:space="preserve">#3f8cff</x:t>
         </x:is>
       </x:c>
+      <x:c r="L4" t="str">
+        <x:v>https://www.corsair.com/ww/de/p/custom-liquid-cooling/cx-9060010-ww/hydro-x-series-xl8-performance-coolant-1l-aca-a-blue-cx-9060010-ww</x:v>
+      </x:c>
+      <x:c r="M4" t="str"/>
+      <x:c r="N4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>CX-9060010-WW</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -2064,6 +2238,10 @@
           <x:t xml:space="preserve">#ee4860</x:t>
         </x:is>
       </x:c>
+      <x:c r="L5" t="str"/>
+      <x:c r="M5" t="str"/>
+      <x:c r="N5" t="str"/>
+      <x:c r="O5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7279,6 +7457,12 @@
     <x:col min="14" max="14" width="24" customWidth="1"/>
     <x:col min="15" max="15" width="24" customWidth="1"/>
     <x:col min="16" max="16" width="24" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="54" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="54" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="54" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -7362,6 +7546,24 @@
           <x:t xml:space="preserve">size</x:t>
         </x:is>
       </x:c>
+      <x:c r="Q1" s="7" t="str">
+        <x:v>maxGpuWithFront360</x:v>
+      </x:c>
+      <x:c r="R1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="S1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
+      <x:c r="T1" s="7" t="str">
+        <x:v>manualUrl</x:v>
+      </x:c>
+      <x:c r="U1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
+      <x:c r="V1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -7447,6 +7649,22 @@
           <x:t xml:space="preserve">Midi-Tower</x:t>
         </x:is>
       </x:c>
+      <x:c r="Q2" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="R2" t="str">
+        <x:v>https://www.fractal-design.com/products/cases/north/north/</x:v>
+      </x:c>
+      <x:c r="S2" t="str">
+        <x:v>https://www.fractal-design.com/app/uploads/2022/12/North_Product-Sheet_EN.pdf</x:v>
+      </x:c>
+      <x:c r="T2" t="str">
+        <x:v>https://www.fractal-design.com/app/uploads/2022/12/North-Manual-V1.2.pdf</x:v>
+      </x:c>
+      <x:c r="U2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="V2" t="str"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -7532,6 +7750,18 @@
           <x:t xml:space="preserve">Midi-Tower</x:t>
         </x:is>
       </x:c>
+      <x:c r="Q3" t="str"/>
+      <x:c r="R3" t="str">
+        <x:v>https://www.corsair.com/de/de/p/pc-cases/cc-9011200-ww/4000d-airflow-tempered-glass-mid-tower-atx-case-black-cc-9011200-ww</x:v>
+      </x:c>
+      <x:c r="S3" t="str"/>
+      <x:c r="T3" t="str"/>
+      <x:c r="U3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="V3" t="str">
+        <x:v>CC-9011200-WW</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -7616,6 +7846,16 @@
           <x:t xml:space="preserve">Micro-Tower</x:t>
         </x:is>
       </x:c>
+      <x:c r="Q4" t="str"/>
+      <x:c r="R4" t="str">
+        <x:v>https://www.asus.com/motherboards-components/cases/prime/asus-prime-ap201-microatx-case/techspec/</x:v>
+      </x:c>
+      <x:c r="S4" t="str"/>
+      <x:c r="T4" t="str"/>
+      <x:c r="U4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="V4" t="str"/>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -7698,6 +7938,16 @@
           <x:t xml:space="preserve">Mini-ITX</x:t>
         </x:is>
       </x:c>
+      <x:c r="Q5" t="str"/>
+      <x:c r="R5" t="str">
+        <x:v>https://www.coolermaster.com/en-global/products/masterbox-nr200p-v2.html</x:v>
+      </x:c>
+      <x:c r="S5" t="str"/>
+      <x:c r="T5" t="str"/>
+      <x:c r="U5" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="V5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7723,6 +7973,9 @@
     <x:col min="13" max="13" width="24" customWidth="1"/>
     <x:col min="14" max="14" width="24" customWidth="1"/>
     <x:col min="15" max="15" width="24" customWidth="1"/>
+    <x:col min="16" max="16" width="54" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="54" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -7801,6 +8054,15 @@
           <x:t xml:space="preserve">standoff</x:t>
         </x:is>
       </x:c>
+      <x:c r="P1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="Q1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
+      <x:c r="R1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -7870,6 +8132,15 @@
       <x:c r="O2" s="2">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="P2" t="str">
+        <x:v>https://www.msi.com/Motherboard/MAG-X870-TOMAHAWK-WIFI/Specification</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>https://storage-asset.msi.com/datasheet/mb/de/MAG-X870-TOMAHAWK-WIFI.pdf</x:v>
+      </x:c>
+      <x:c r="R2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -7939,6 +8210,13 @@
       <x:c r="O3" s="2">
         <x:v>8</x:v>
       </x:c>
+      <x:c r="P3" t="str">
+        <x:v>https://www.asrock.com/mb/amd/B850M%20Pro%20RS%20WiFi/</x:v>
+      </x:c>
+      <x:c r="Q3" t="str"/>
+      <x:c r="R3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -8008,6 +8286,13 @@
       <x:c r="O4" s="2">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="P4" t="str">
+        <x:v>https://www.gigabyte.com/Motherboard/Z890-AORUS-ELITE-WIFI7/sp</x:v>
+      </x:c>
+      <x:c r="Q4" t="str"/>
+      <x:c r="R4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -8077,6 +8362,13 @@
       <x:c r="O5" s="2">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="P5" t="str">
+        <x:v>https://rog.asus.com/de/motherboards/rog-strix/rog-strix-b860-i-gaming-wifi/spec/</x:v>
+      </x:c>
+      <x:c r="Q5" t="str"/>
+      <x:c r="R5" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
@@ -8144,6 +8436,13 @@
       <x:c r="O6" s="2">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="P6" t="str">
+        <x:v>https://www.msi.com/Motherboard/B650-GAMING-PLUS-WIFI/Specification</x:v>
+      </x:c>
+      <x:c r="Q6" t="str"/>
+      <x:c r="R6" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="2" t="inlineStr">
@@ -8211,6 +8510,13 @@
       <x:c r="O7" s="2">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="P7" t="str">
+        <x:v>https://www.msi.com/Motherboard/PRO-Z790-P-WIFI-DDR4/Specification</x:v>
+      </x:c>
+      <x:c r="Q7" t="str"/>
+      <x:c r="R7" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="2" t="inlineStr">
@@ -8277,6 +8583,13 @@
       </x:c>
       <x:c r="O8" s="2">
         <x:v>8</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>https://www.msi.com/Motherboard/B550M-PRO-VDH-WIFI/Specification</x:v>
+      </x:c>
+      <x:c r="Q8" t="str"/>
+      <x:c r="R8" t="str">
+        <x:v>2026-09-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8300,6 +8613,8 @@
     <x:col min="10" max="10" width="24" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
     <x:col min="12" max="12" width="24" customWidth="1"/>
+    <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -8363,6 +8678,12 @@
           <x:t xml:space="preserve">label</x:t>
         </x:is>
       </x:c>
+      <x:c r="M1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -8421,6 +8742,12 @@
           <x:t xml:space="preserve">R5</x:t>
         </x:is>
       </x:c>
+      <x:c r="M2" t="str">
+        <x:v>https://www.amd.com/en/products/processors/desktops/ryzen/9000-series/amd-ryzen-5-9600x.html</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -8479,6 +8806,12 @@
           <x:t xml:space="preserve">R7</x:t>
         </x:is>
       </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://www.amd.com/de/products/processors/desktops/ryzen/9000-series/amd-ryzen-7-9800x3d.html</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -8537,6 +8870,12 @@
           <x:t xml:space="preserve">R9</x:t>
         </x:is>
       </x:c>
+      <x:c r="M4" t="str">
+        <x:v>https://www.amd.com/en/products/processors/desktops/ryzen/9000-series/amd-ryzen-9-9950x3d.html</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -8595,6 +8934,12 @@
           <x:t xml:space="preserve">U5</x:t>
         </x:is>
       </x:c>
+      <x:c r="M5" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/241067/intel-core-ultra-5-processor-245k-24m-cache-up-to-5-20-ghz/specifications.html</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
@@ -8653,6 +8998,12 @@
           <x:t xml:space="preserve">U7</x:t>
         </x:is>
       </x:c>
+      <x:c r="M6" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/241063/intel-core-ultra-7-processor-265k-30m-cache-up-to-5-50-ghz/specifications.html</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="2" t="inlineStr">
@@ -8711,6 +9062,12 @@
           <x:t xml:space="preserve">U9</x:t>
         </x:is>
       </x:c>
+      <x:c r="M7" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/241060/intel-core-ultra-9-processor-285k-36m-cache-up-to-5-70-ghz/specifications.html</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="2" t="inlineStr">
@@ -8767,6 +9124,12 @@
           <x:t xml:space="preserve">R5</x:t>
         </x:is>
       </x:c>
+      <x:c r="M8" t="str">
+        <x:v>https://www.amd.com/en/products/processors/desktops/ryzen/7000-series/amd-ryzen-5-7600.html</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="2" t="inlineStr">
@@ -8823,6 +9186,12 @@
           <x:t xml:space="preserve">R7</x:t>
         </x:is>
       </x:c>
+      <x:c r="M9" t="str">
+        <x:v>https://www.amd.com/en/products/processors/desktops/ryzen/7000-series/amd-ryzen-7-7800x3d.html</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="2" t="inlineStr">
@@ -8879,6 +9248,12 @@
           <x:t xml:space="preserve">i5</x:t>
         </x:is>
       </x:c>
+      <x:c r="M10" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/236799/intel-core-i5-processor-14600k-24m-cache-up-to-5-30-ghz/specifications.html</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="2" t="inlineStr">
@@ -8935,6 +9310,12 @@
           <x:t xml:space="preserve">R7</x:t>
         </x:is>
       </x:c>
+      <x:c r="M11" t="str">
+        <x:v>https://www.amd.com/en/products/processors/desktops/ryzen/5000-series/amd-ryzen-7-5800x3d.html</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="2" t="inlineStr">
@@ -8990,6 +9371,12 @@
         <x:is>
           <x:t xml:space="preserve">i7</x:t>
         </x:is>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/134594/intel-core-i712700k-processor-25m-cache-up-to-5-00-ghz/specifications.html</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>2026-09-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9013,582 +9400,538 @@
     <x:col min="10" max="10" width="24" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
     <x:col min="12" max="12" width="24" customWidth="1"/>
+    <x:col min="15" max="15" width="54" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="54" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="54" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="19" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">maker</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">price</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">generation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">recommended</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">beginnerVariant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">specs</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">length</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">power</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">connector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">label</x:t>
-        </x:is>
+      <x:c r="A1" s="1" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="str">
+        <x:v>maker</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="str">
+        <x:v>price</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="str">
+        <x:v>generation</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="str">
+        <x:v>recommended</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="str">
+        <x:v>beginnerVariant</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="str">
+        <x:v>specs</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="str">
+        <x:v>length</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="str">
+        <x:v>power</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="str">
+        <x:v>connector</x:v>
+      </x:c>
+      <x:c r="L1" s="1" t="str">
+        <x:v>label</x:v>
+      </x:c>
+      <x:c r="M1" s="7" t="str">
+        <x:v>chipMaker</x:v>
+      </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
+      <x:c r="O1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="P1" s="7" t="str">
+        <x:v>gpuFamilyUrl</x:v>
+      </x:c>
+      <x:c r="Q1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
+      <x:c r="R1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
-      <x:c r="A2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5060ti</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NVIDIA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GeForce RTX 5060 Ti 16 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D2" s="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>5060ti</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>MSI</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>MSI GeForce RTX 5060 Ti 16G VENTUS 2X OC PLUS</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="n">
         <x:v>499</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">true</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">a</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 GB GDDR7
+      <x:c r="E2" s="2" t="str"/>
+      <x:c r="F2" s="2" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>16 GB GDDR7
+227 mm
+180 W</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="n">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="str">
+        <x:v>8-pin</x:v>
+      </x:c>
+      <x:c r="L2" s="2" t="str">
+        <x:v>5060 Ti</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>G506T-16V2CP</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>https://www.msi.com/Graphics-Card/GeForce-RTX-5060-Ti-16G-VENTUS-2X-OC-PLUS/Specification</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>https://www.nvidia.com/de-de/geforce/graphics-cards/50-series/rtx-5060-family/</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>https://storage-asset.msi.com/datasheet/vga/global/GeForce-RTX-5060-Ti-16G-VENTUS-2X-OC-PLUS.pdf</x:v>
+      </x:c>
+      <x:c r="R2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="48" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>5070</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>MSI</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>MSI GeForce RTX 5070 12G VENTUS 2X OC</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="n">
+        <x:v>649</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str"/>
+      <x:c r="F3" s="2" t="str"/>
+      <x:c r="G3" s="2" t="str"/>
+      <x:c r="H3" s="2" t="str">
+        <x:v>12 GB GDDR7
+236 mm
+250 W</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="n">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="J3" s="2" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="str">
+        <x:v>16-pin</x:v>
+      </x:c>
+      <x:c r="L3" s="2" t="str">
+        <x:v>RTX 5070</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>G5070-12V2C</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>https://www.msi.com/Graphics-Card/GeForce-RTX-5070-12G-VENTUS-2X-OC/Specification</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>https://www.nvidia.com/de-de/geforce/graphics-cards/50-series/rtx-5070-family/</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>https://storage-asset.msi.com/datasheet/vga/global/GeForce-RTX-5070-12G-VENTUS-2X-OC.pdf</x:v>
+      </x:c>
+      <x:c r="R3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
+      <x:c r="A4" s="2" t="str">
+        <x:v>5080</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>MSI</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>MSI GeForce RTX 5080 16G VENTUS 3X OC</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="n">
+        <x:v>1199</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str"/>
+      <x:c r="F4" s="2" t="str"/>
+      <x:c r="G4" s="2" t="str"/>
+      <x:c r="H4" s="2" t="str">
+        <x:v>16 GB GDDR7
+303 mm
+360 W</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="n">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="J4" s="2" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="K4" s="2" t="str">
+        <x:v>16-pin</x:v>
+      </x:c>
+      <x:c r="L4" s="2" t="str">
+        <x:v>RTX 5080</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>G5080-16V3C</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>https://de.msi.com/Graphics-Card/GeForce-RTX-5080-16G-VENTUS-3X-OC/Specification</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>https://www.nvidia.com/de-de/geforce/graphics-cards/50-series/rtx-5080/</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>https://storage-asset.msi.com/datasheet/vga/de/GeForce-RTX-5080-16G-VENTUS-3X-OC.pdf</x:v>
+      </x:c>
+      <x:c r="R4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>9070</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>Sapphire</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>Sapphire PULSE Radeon RX 9070 16G</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="n">
+        <x:v>659</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str"/>
+      <x:c r="F5" s="2" t="str"/>
+      <x:c r="G5" s="2" t="str"/>
+      <x:c r="H5" s="2" t="str">
+        <x:v>16 GB GDDR6
+280 mm
+220 W</x:v>
+      </x:c>
+      <x:c r="I5" s="2" t="n">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="J5" s="2" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="K5" s="2" t="str">
+        <x:v>2× 8-pin</x:v>
+      </x:c>
+      <x:c r="L5" s="2" t="str">
+        <x:v>RX 9070</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>AMD</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>11349-03-20G</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>https://www.sapphiretech.com/en/consumer/pulse-radeon-rx-9070-16g-gddr6</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>https://www.amd.com/en/products/graphics/desktops/radeon/9000-series/amd-radeon-rx-9070.html</x:v>
+      </x:c>
+      <x:c r="Q5" t="str"/>
+      <x:c r="R5" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>9070xt</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>Sapphire</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>Sapphire PULSE Radeon RX 9070 XT 16G</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="n">
+        <x:v>759</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str"/>
+      <x:c r="F6" s="2" t="str"/>
+      <x:c r="G6" s="2" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="H6" s="2" t="str">
+        <x:v>16 GB GDDR6
+320 mm
+304 W</x:v>
+      </x:c>
+      <x:c r="I6" s="2" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="J6" s="2" t="n">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="K6" s="2" t="str">
+        <x:v>2× 8-pin</x:v>
+      </x:c>
+      <x:c r="L6" s="2" t="str">
+        <x:v>9070 XT</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>AMD</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>11348-03-20G</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>https://www.sapphiretech.com/en/consumer/pulse-radeon-rx-9070-xt-16g-gddr6</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>https://www.amd.com/de/products/graphics/desktops/radeon/9000-series/amd-radeon-rx-9070xt.html</x:v>
+      </x:c>
+      <x:c r="Q6" t="str"/>
+      <x:c r="R6" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>4070super</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>MSI</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>MSI GeForce RTX 4070 SUPER 12G VENTUS 2X OC</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="n">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="str"/>
+      <x:c r="G7" s="2" t="str"/>
+      <x:c r="H7" s="2" t="str">
+        <x:v>12 GB GDDR6X
 242 mm
-180 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I2" s="2">
+220 W</x:v>
+      </x:c>
+      <x:c r="I7" s="2" t="n">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="J2" s="2">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="K2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8-pin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5060 Ti</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="48" customHeight="1">
-      <x:c r="A3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5070</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NVIDIA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GeForce RTX 5070 12 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="2">
-        <x:v>649</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12 GB GDDR7
-242 mm
-250 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I3" s="2">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="J3" s="2">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="K3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12V-2x6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RTX 5070</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="48" customHeight="1">
-      <x:c r="A4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5080</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NVIDIA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GeForce RTX 5080 16 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="2">
-        <x:v>1199</x:v>
-      </x:c>
-      <x:c r="E4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 GB GDDR7
-304 mm
-360 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I4" s="2">
-        <x:v>304</x:v>
-      </x:c>
-      <x:c r="J4" s="2">
-        <x:v>360</x:v>
-      </x:c>
-      <x:c r="K4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12V-2x6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RTX 5080</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="48" customHeight="1">
-      <x:c r="A5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">9070</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AMD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Radeon RX 9070 16 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="2">
-        <x:v>659</x:v>
-      </x:c>
-      <x:c r="E5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 GB GDDR6
-289 mm
-220 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I5" s="2">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J5" s="2">
+      <x:c r="J7" s="2" t="n">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="K5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2× 8-pin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RX 9070</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">9070xt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AMD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Radeon RX 9070 XT 16 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="2">
-        <x:v>759</x:v>
-      </x:c>
-      <x:c r="E6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">b</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 GB GDDR6
-304 mm
-304 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I6" s="2">
-        <x:v>304</x:v>
-      </x:c>
-      <x:c r="J6" s="2">
-        <x:v>304</x:v>
-      </x:c>
-      <x:c r="K6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3× 8-pin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">9070 XT</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="48" customHeight="1">
-      <x:c r="A7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4070super</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NVIDIA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GeForce RTX 4070 SUPER 12 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="2">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="E7" s="2">
+      <x:c r="K7" s="2" t="str">
+        <x:v>16-pin</x:v>
+      </x:c>
+      <x:c r="L7" s="2" t="str">
+        <x:v>4070 S</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="N7" t="str"/>
+      <x:c r="O7" t="str">
+        <x:v>https://www.msi.com/Graphics-Card/GeForce-RTX-4070-SUPER-12G-VENTUS-2X-OC/Specification</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>https://www.nvidia.com/de-de/geforce/graphics-cards/40-series/rtx-4070-family/</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>https://storage-asset.msi.com/datasheet/vga/global/GeForce-RTX-4070-SUPER-12G-VENTUS-2X-OC.pdf</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>7800xt</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>Sapphire</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>Sapphire Radeon RX 7800 XT 16G</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="n">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12 GB GDDR6X
+      <x:c r="F8" s="2" t="str"/>
+      <x:c r="G8" s="2" t="str"/>
+      <x:c r="H8" s="2" t="str">
+        <x:v>16 GB GDDR6
 267 mm
-220 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I7" s="2">
+263 W</x:v>
+      </x:c>
+      <x:c r="I8" s="2" t="n">
         <x:v>267</x:v>
       </x:c>
-      <x:c r="J7" s="2">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="K7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12V-2x6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4070 S</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="48" customHeight="1">
-      <x:c r="A8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">7800xt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AMD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Radeon RX 7800 XT 16 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" s="2">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="E8" s="2">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 GB GDDR6
+      <x:c r="J8" s="2" t="n">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="K8" s="2" t="str">
+        <x:v>2× 8-pin</x:v>
+      </x:c>
+      <x:c r="L8" s="2" t="str">
+        <x:v>7800 XT</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>AMD</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>21330-01-20G</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>https://www.sapphiretech.com/en/consumer/21330-01-20g-radeon-rx-7800-xt-16g-gddr6</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>https://www.amd.com/de/products/graphics/desktops/radeon/7000-series/amd-radeon-rx-7800-xt.html</x:v>
+      </x:c>
+      <x:c r="Q8" t="str"/>
+      <x:c r="R8" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>3080</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>MSI</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>MSI GeForce RTX 3080 VENTUS 3X 10G OC</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="n">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="str"/>
+      <x:c r="G9" s="2" t="str"/>
+      <x:c r="H9" s="2" t="str">
+        <x:v>10 GB GDDR6X
+305 mm
+320 W</x:v>
+      </x:c>
+      <x:c r="I9" s="2" t="n">
+        <x:v>305</x:v>
+      </x:c>
+      <x:c r="J9" s="2" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="K9" s="2" t="str">
+        <x:v>2× 8-pin</x:v>
+      </x:c>
+      <x:c r="L9" s="2" t="str">
+        <x:v>RTX 3080</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="N9" t="str"/>
+      <x:c r="O9" t="str">
+        <x:v>https://de.msi.com/Graphics-Card/GeForce-RTX-3080-VENTUS-3X-10G-OC/Specification</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>https://www.nvidia.com/de-de/geforce/graphics-cards/30-series/rtx-3080-3080ti/</x:v>
+      </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>https://storage-asset.msi.com/datasheet/vga/de/GeForce-RTX-3080-VENTUS-3X-10G-OC.pdf</x:v>
+      </x:c>
+      <x:c r="R9" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>6800xt</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Sapphire</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>Sapphire Radeon RX 6800 XT 16G</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="n">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str"/>
+      <x:c r="G10" s="2" t="str"/>
+      <x:c r="H10" s="2" t="str">
+        <x:v>16 GB GDDR6
 267 mm
-263 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I8" s="2">
+300 W</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="n">
         <x:v>267</x:v>
       </x:c>
-      <x:c r="J8" s="2">
-        <x:v>263</x:v>
-      </x:c>
-      <x:c r="K8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2× 8-pin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L8" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">7800 XT</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3080</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NVIDIA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GeForce RTX 3080 10 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" s="2">
-        <x:v>349</x:v>
-      </x:c>
-      <x:c r="E9" s="2">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10 GB GDDR6X
-285 mm
-320 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I9" s="2">
-        <x:v>285</x:v>
-      </x:c>
-      <x:c r="J9" s="2">
-        <x:v>320</x:v>
-      </x:c>
-      <x:c r="K9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2× 8-pin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RTX 3080</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="48" customHeight="1">
-      <x:c r="A10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6800xt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AMD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Radeon RX 6800 XT 16 GB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="2">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="E10" s="2">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 GB GDDR6
-267 mm
-300 W</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I10" s="2">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="J10" s="2">
+      <x:c r="J10" s="2" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="K10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2× 8-pin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6800 XT</x:t>
-        </x:is>
+      <x:c r="K10" s="2" t="str">
+        <x:v>2× 8-pin</x:v>
+      </x:c>
+      <x:c r="L10" s="2" t="str">
+        <x:v>6800 XT</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>AMD</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>21304-01-20G</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>https://nation.sapphiretech.com/en/consumer/21304-01-20g-radeon-rx-6800-xt-16g-gddr6</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>https://www.amd.com/en/products/graphics/desktops/radeon/6000-series/amd-radeon-rx-6800-xt.html</x:v>
+      </x:c>
+      <x:c r="Q10" t="str"/>
+      <x:c r="R10" t="str">
+        <x:v>2026-09-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9612,6 +9955,10 @@
     <x:col min="10" max="10" width="24" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
     <x:col min="12" max="12" width="24" customWidth="1"/>
+    <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -9675,6 +10022,18 @@
           <x:t xml:space="preserve">speed</x:t>
         </x:is>
       </x:c>
+      <x:c r="M1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
+      <x:c r="O1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
+      <x:c r="P1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -9731,6 +10090,16 @@
       <x:c r="L2" s="2">
         <x:v>6000</x:v>
       </x:c>
+      <x:c r="M2" t="str">
+        <x:v>https://www.gskill.com/specification/165/396/1673491242/F5-6000J3038F16GX2-FX5-Specification</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>F5-6000J3038F16GX2-FX5</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="P2" t="str"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -9787,6 +10156,18 @@
       <x:c r="L3" s="2">
         <x:v>6000</x:v>
       </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://www.kingston.com/de/memory/search/discontinuedmodels?partid=KF560C30BBK2-64</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>KF560C30BBK2-64</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>https://www.kingston.com/datasheets/KF560C30BBK2-64.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -9843,6 +10224,16 @@
       <x:c r="L4" s="2">
         <x:v>6400</x:v>
       </x:c>
+      <x:c r="M4" t="str">
+        <x:v>https://www.corsair.com/de/de/p/memory/cmh64gx5m2b6400c32/vengeance-rgb-64gb-2x32gb-ddr5-dram-6400mts-c32-memory-kit-black-cmh64gx5m2b6400c32</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>CMH64GX5M2B6400C32</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="P4" t="str"/>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -9899,6 +10290,10 @@
       <x:c r="L5" s="2">
         <x:v>6400</x:v>
       </x:c>
+      <x:c r="M5" t="str"/>
+      <x:c r="N5" t="str"/>
+      <x:c r="O5" t="str"/>
+      <x:c r="P5" t="str"/>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
@@ -9953,6 +10348,16 @@
       <x:c r="L6" s="2">
         <x:v>3600</x:v>
       </x:c>
+      <x:c r="M6" t="str">
+        <x:v>https://www.gskill.com/tw/specification/203/217/1562831784/F4-3600C16D-32GVKC-Specification</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>F4-3600C16D-32GVKC</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="P6" t="str"/>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="2" t="inlineStr">
@@ -10007,6 +10412,16 @@
       <x:c r="L7" s="2">
         <x:v>3200</x:v>
       </x:c>
+      <x:c r="M7" t="str">
+        <x:v>https://www.kingston.com/de/memory/search?partid=KF432C16BBK2%2F64</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>KF432C16BBK2/64</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="P7" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10028,6 +10443,9 @@
     <x:col min="9" max="9" width="24" customWidth="1"/>
     <x:col min="10" max="10" width="24" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
+    <x:col min="12" max="12" width="54" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -10086,6 +10504,15 @@
           <x:t xml:space="preserve">atx3</x:t>
         </x:is>
       </x:c>
+      <x:c r="L1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="M1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -10141,6 +10568,15 @@
           <x:t xml:space="preserve">true</x:t>
         </x:is>
       </x:c>
+      <x:c r="L2" t="str">
+        <x:v>https://www.corsair.com/ww/de/p/psu/cp-9020302-ww/rme-series-rm650e-fully-modular-low-noise-atx-power-supply-ww-cp-9020302-ww</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>CP-9020302-WW</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -10196,6 +10632,13 @@
           <x:t xml:space="preserve">true</x:t>
         </x:is>
       </x:c>
+      <x:c r="L3" t="str">
+        <x:v>https://www.bequiet.com/de/powersupply/4068</x:v>
+      </x:c>
+      <x:c r="M3" t="str"/>
+      <x:c r="N3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -10251,6 +10694,15 @@
           <x:t xml:space="preserve">true</x:t>
         </x:is>
       </x:c>
+      <x:c r="L4" t="str">
+        <x:v>https://www.corsair.com/eu/de/p/psu/cp-9020270-eu/rmx-series-rm850x-fully-modular-power-supply-eu-cp-9020270-eu</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>CP-9020270-EU</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -10306,6 +10758,9 @@
           <x:t xml:space="preserve">true</x:t>
         </x:is>
       </x:c>
+      <x:c r="L5" t="str"/>
+      <x:c r="M5" t="str"/>
+      <x:c r="N5" t="str"/>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
@@ -10361,6 +10816,13 @@
           <x:t xml:space="preserve">true</x:t>
         </x:is>
       </x:c>
+      <x:c r="L6" t="str">
+        <x:v>https://www.coolermaster.com/de-de/products/v750-sfx-gold.html</x:v>
+      </x:c>
+      <x:c r="M6" t="str"/>
+      <x:c r="N6" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="2" t="inlineStr">
@@ -10414,6 +10876,9 @@
           <x:t xml:space="preserve">false</x:t>
         </x:is>
       </x:c>
+      <x:c r="L7" t="str"/>
+      <x:c r="M7" t="str"/>
+      <x:c r="N7" t="str"/>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="2" t="inlineStr">
@@ -10467,6 +10932,9 @@
           <x:t xml:space="preserve">false</x:t>
         </x:is>
       </x:c>
+      <x:c r="L8" t="str"/>
+      <x:c r="M8" t="str"/>
+      <x:c r="N8" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10490,6 +10958,10 @@
     <x:col min="11" max="11" width="24" customWidth="1"/>
     <x:col min="12" max="12" width="38" customWidth="1"/>
     <x:col min="13" max="13" width="24" customWidth="1"/>
+    <x:col min="14" max="14" width="54" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="54" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -10558,6 +11030,18 @@
           <x:t xml:space="preserve">radiator</x:t>
         </x:is>
       </x:c>
+      <x:c r="N1" s="7" t="str">
+        <x:v>sourceUrl</x:v>
+      </x:c>
+      <x:c r="O1" s="7" t="str">
+        <x:v>datasheetUrl</x:v>
+      </x:c>
+      <x:c r="P1" s="7" t="str">
+        <x:v>modelNumber</x:v>
+      </x:c>
+      <x:c r="Q1" s="7" t="str">
+        <x:v>sourceCheckedAt</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="inlineStr">
@@ -10624,6 +11108,18 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
+      <x:c r="N2" t="str">
+        <x:v>https://www.arctic.de/en/Freezer-36/ACFRE00121A</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>https://www.arctic.de/media/6b/50/57/1709195123/Spec_Sheet_Freezer_36_EN.pdf</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>ACFRE00121A</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="inlineStr">
@@ -10690,6 +11186,16 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
+      <x:c r="N3" t="str">
+        <x:v>https://www.noctua.at/en/products/nh-d15-g2/specifications</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>https://noctua.at/pub/media/blfa_files/infosheet/noctua_nh_d15_g2_datasheet_de_web_1.pdf</x:v>
+      </x:c>
+      <x:c r="P3" t="str"/>
+      <x:c r="Q3" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="inlineStr">
@@ -10756,6 +11262,18 @@
       <x:c r="M4" s="2">
         <x:v>240</x:v>
       </x:c>
+      <x:c r="N4" t="str">
+        <x:v>https://www.arctic.de/en/Liquid-Freezer-III-240/ACFRE00134A</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>https://www.arctic.de/media/1c/af/b3/1708429821/Spec_Sheet_Liquid_Freezer_III_240_Black_EN.pdf</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>ACFRE00134A</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
@@ -10822,6 +11340,14 @@
       <x:c r="M5" s="2">
         <x:v>360</x:v>
       </x:c>
+      <x:c r="N5" t="str">
+        <x:v>https://www.arctic.de/en/Liquid-Freezer-III-360/ACFRE00136A</x:v>
+      </x:c>
+      <x:c r="O5" t="str"/>
+      <x:c r="P5" t="str"/>
+      <x:c r="Q5" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
@@ -10888,6 +11414,10 @@
       <x:c r="M6" s="2">
         <x:v>360</x:v>
       </x:c>
+      <x:c r="N6" t="str"/>
+      <x:c r="O6" t="str"/>
+      <x:c r="P6" t="str"/>
+      <x:c r="Q6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>